<commit_message>
Print the handler code down the sheet instead of inside one wide cell
It was there - 477 to 2,055 characters per cell - and it read as empty:
column F sits past five wide columns, so it is off the side of the screen,
and a fixed 150pt row height clips a 90-line method to about ten lines.
Shipping code in a wrapped cell was the wrong call.

The Handler code sheet is now one line of ABAP per row down column A, in
Consolas, with a dark bar naming the journey, ticket and class above each
block. Nothing wraps, nothing is clipped, and it copies out as code rather
than as one run-on string. 459 rows across the eleven fixes.

The same snippets are also written to doc/tickets/handler_code/*.abap, one
file per fix, for anyone who would rather open a file than a spreadsheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VWo9ZYCDErS8LYrKBBSZ5R
</commit_message>
<xml_diff>
--- a/doc/tickets/CJS_journey_ownership.xlsx
+++ b/doc/tickets/CJS_journey_ownership.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +55,19 @@
       <name val="Consolas"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +119,11 @@
         <fgColor rgb="00F6DDE1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EEED"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -126,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,7 +197,11 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -9350,15 +9370,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:A459"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="120" customWidth="1" min="6" max="6"/>
+    <col width="118" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9369,749 +9384,2903 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>These are the journey's OWN class, not the framework. Read it, take it or write your own - it is your service. Where a whole method is given, it is the complete current method: replace the method body with it. Nothing here is pushed for you.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Journey</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Method / where</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>What it fixes</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="150" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>E025</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-703</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E025_BEEKEEPING_LOGIC</t>
-        </is>
-      </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>see the code</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Applicant BP was written to the owner SEARCH field and then blanked</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>* --- private section: the constant named the wrong field ------------
-*   was:  constants C_LOGIN_BP type STRING value 'OWNER_BP' ##NO_TEXT.
-  constants C_LOGIN_BP type STRING value 'LOGIN_BP' ##NO_TEXT.
-* --- ZIF_RAK_JOURNEY_LOGIC~ON_INIT, last line inside the IF -----------
-*   was:  io_ctx-&gt;set_val( iv_name = 'OWNER_BP' iv_value = ' ' ).
-*   'OWNER_BP' is the owner search box (see ON_SEARCH), not the applicant.
-  io_ctx-&gt;set_val( iv_name = c_owner_bp iv_value = ' ' ).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="150" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>E026</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-704</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E026_TREE_REMOVAL_LOGIC</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>see the code</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Applicant BP never reached LOGIN_BP</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>* --- private section: add, leave C_LOGIN_BP exactly as it is ---------
-  constants C_APP_BP type STRING value 'LOGIN_BP' ##NO_TEXT.
-* --- ZIF_RAK_JOURNEY_LOGIC~ON_INIT, straight after the existing line --
-    io_ctx-&gt;set_val( iv_name = c_login_bp iv_value = |{ lv_loginbp }| ).
-    io_ctx-&gt;set_val( iv_name = c_app_bp   iv_value = |{ lv_loginbp }| ).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="150" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>E018</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-697</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>see the code</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>The class had NO ACTIVE VERSION - a string constant does not take an empty literal, so every earlier fix was in the source and none of it was running</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>* --- private section --------------------------------------------------
-*   was:  constants C_IMPEXP type STRING value ''.       &lt;- will not compile
-  constants C_IMPEXP type STRING value IS INITIAL ##NO_TEXT.
-* Activate the class after this and re-test the whole journey - including the
-* CX_SY_CONVERSION_NO_NUMBER on post, which may go with it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>E022</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-684</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_EPDA_E022_DEV_PROJ_LOGIC</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_INIT</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Applicant details were written twice on ON_INIT</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_init.
-*CALL METHOD SUPER-&gt;ZIF_RAK_JOURNEY_LOGIC~ON_INIT
-*  EXPORTING
-*    IO_CTX =
-*    .
-    CALL METHOD super-&gt;zif_rak_journey_logic~on_init
-      EXPORTING
-        io_ctx = io_ctx.
-    DATA: lv_loginbp TYPE bu_partner.
-    lv_loginbp       = CAST zcl_rak_journey_engine( io_ctx )-&gt;mv_loginbp.
-    DATA(lv_rolebp)  = CAST zcl_rak_journey_engine( io_ctx )-&gt;mv_rolebp.
-    DATA(lv_role)    = CAST zcl_rak_journey_engine( io_ctx )-&gt;mv_role. "Owner
-    IF lv_loginbp IS NOT INITIAL.
-      NEW zcl_ega_epda_fshry_handler_api( )-&gt;get_bp_details(
-        EXPORTING
-          iv_bp_id      = lv_loginbp
-        IMPORTING
-          es_bp_details = DATA(ls_bp) ).
-      io_ctx-&gt;set_val( iv_name = c_login_bp iv_value = |{ lv_loginbp }| ).
-*     WRITTEN ONCE. C_PARTNER_NAME is 'APP_NAME' and C_PARTNER_ID is
-*     'APP_ID', and both were then written a SECOND time below this IF, under
-*     a different language rule - so the two disagreed and the later one won.
-*     The pair below the IF was also outside this guard, so a launch with no
-*     login partner blanked the applicant's name and ID rather than leaving
-*     them alone.
-*
-*     The rule kept is the one that degrades: an Arabic session with no
-*     Arabic name on the partner record falls back to the English name
-*     rather than showing an empty applicant.
-      io_ctx-&gt;set_val( iv_name  = c_partner_name
-                       iv_value = COND #( WHEN sy-langu &lt;&gt; c_lang_en AND ls_bp-bp_name_ar IS NOT INITIAL
-                                          THEN CONV string( ls_bp-bp_name_ar )
-                                          ELSE CONV string( ls_bp-bp_name ) ) ).
-      io_ctx-&gt;set_val( iv_name = c_partner_id iv_value = CONV #( ls_bp-emirates_id ) ).
-      io_ctx-&gt;set_val( iv_name = c_partner_mobile iv_value = CONV #( ls_bp-mobile_number ) ).
-      io_ctx-&gt;set_val( iv_name = c_partner_email iv_value = CONV #( ls_bp-email_address ) ).
-      io_ctx-&gt;set_val( iv_name = c_applicanttype iv_value = |{ lv_role }| ).
-    ENDIF.
-  ENDMETHOD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="150" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>E022 E026 E027 D021 D014gv</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-684 / 704</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>six classes - see the code</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>see the code</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>The applicant's own partner never reached LOGIN_BP, the field every other journey and the record model use. Additive: the existing OWNER_BP write is left alone, so nothing that works today changes</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>* Applies to ZCL_EPDA_E022_DEV_PROJ_LOGIC, ZCL_E026_TREE_REMOVAL_LOGIC,
-* ZCL_E027_VICE_CAPTAIN_LOGIC, ZCL_D021_MOD_SCHOOL_FEE_LOGIC and
-* ZCL_D014_STAFF_GOLD_VISA_LOGIC - all five declare C_LOGIN_BP as 'OWNER_BP'.
-* E025 is the exception and has its own row above: there OWNER_BP is the owner
-* SEARCH box, so the constant itself has to be corrected, not added to.
-* --- private section: ADD this. Leave C_LOGIN_BP exactly as it is. ----
-  constants C_APP_BP type STRING value 'LOGIN_BP' ##NO_TEXT.
-* --- ON_INIT: ADD the second line under the existing first one. -------
-    io_ctx-&gt;set_val( iv_name = c_login_bp iv_value = |{ lv_loginbp }| ).
-    io_ctx-&gt;set_val( iv_name = c_app_bp   iv_value = |{ lv_loginbp }| ).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>E017</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-687</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E017_NOC_EXP_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_CUSTOM_VALIDATE</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Step 0 refused whenever the role flags disagreed with APPLICANT_ROLE - re-derived now instead of refused</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_custom_validate.
-    rt = super-&gt;zif_rak_journey_logic~on_custom_validate( io_ctx  = io_ctx
-                                                          iv_step = iv_step ).
-    CASE iv_step.
-      WHEN 0.
-*       RE-DERIVED, NOT REFUSED.
-*
-*       PARTNER_OWNER/PARTNER_REP and PERMIT_YES/PERMIT_NO are not answers
-*       in their own right - they are WRITE_FLAGS( )'s projection of
-*       APPLICANT_ROLE and PERMIT_HELD, which are the fields the citizen
-*       actually fills in. This used to refuse the step whenever the role
-*       was set and its flags were not, with "Re-select Owner or
-*       Representative before continuing."
-*
-*       The citizen had already selected it. WRITE_FLAGS( ) only runs from
-*       ON_CHANGE( ), so any round trip that reinstates the model without
-*       raising a change on APPLICANT_ROLE - a backend read answering the
-*       step, the BP search coming back - leaves the role set and the flags
-*       blank. Re-selecting the same value raises no CHANGE either, so the
-*       one instruction the message gave could not clear it: the journey
-*       stopped at step 1. Reported on all three chemical journeys as
-*       "error showing we u select representative and search with owner EID
-*       details, not moving to next step".
-*
-*       Rewriting them is what the handler does at post time anyway -
-*       ON_BEFORE_POST( ) calls WRITE_FLAGS( ) before every post - so doing
-*       it here costs nothing and removes the only state that could block.
-        write_flags( io_ctx ).
-      WHEN 2.
-        DATA(ls_grid) = io_ctx-&gt;get_grid_data( c_grid ).
-        IF ls_grid-rows IS INITIAL.
-          APPEND VALUE #( type  = 'Error' "field = c_grid
-                          text  = `Add at least one chemical row.` ) TO rt.
-        ENDIF.
-      WHEN OTHERS.
-    ENDCASE.
-  ENDMETHOD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>E017</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-687</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E017_NOC_EXP_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>METHOD VALIDATE_INPUT</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Add Chemical: all fourteen fields enforced. Ten of the checks were commented out</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD validate_input.
-*   ALL FOURTEEN, mirroring the REQUIRED markers in ON_RENDER_POPUP( ).
-*   Ten of these were commented out; CJSMIG-687 Issue 4 settled it.
-    IF io_ctx-&gt;get_val( c_hs_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_mat_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_chem_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_cas_no_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_chem_form_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_packaging_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_quantity_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_gross_weight_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_unit_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_bol_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_exit_port_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_import_pop ) IS INITIAL
-             OR io_ctx-&gt;get_val( c_tport_pop ) IS INITIAL.
-      io_ctx-&gt;add_msg( iv_type = 'Warning'
-                       iv_text = 'Kindly fill required details.' ).
-*     RV_OK stays FALSE. This used to return nothing at all, and ON_POPUP_EVENT
-*     called POPULATE_GRID( ) and CLOSE_POPUP( ) straight afterwards whatever
-*     happened here - so a blank row was added to the grid and the dialog shut,
-*     with only a warning toast to say otherwise. The verdict has to reach the
-*     caller for the message to mean anything.
-      RETURN.
-    ENDIF.
-    rv_ok = abap_true.
-  ENDMETHOD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>E017</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-687</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E017_NOC_EXP_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_RENDER_POPUP</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Add Chemical: the fourteen required markers, and IV_COLUMNS = 2 for the two-column dialog</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_render_popup.
-    super-&gt;zif_rak_journey_logic~on_render_popup(
-      io_ctx   = io_ctx
-      io_popup = io_popup
-      iv_id    = iv_id
-    ).
-    CASE iv_id.
-*  "On click of ADD Chemical button
-      WHEN c_open_popup.
-*        render_own_popup( io_ctx = io_ctx io_popup = io_popup ).
-*        RETURN.
-*       REQUIRED here is the marker only - DIALOG_FORM( ) sets it on the label
-*       and enforces nothing; a popup's enforcement is the handler's, in
-*       VALIDATE_INPUT( ). So this list has to mirror that method exactly,
-*       and now does: all fourteen marked, all fourteen checked.
-*
-*       That mirror used to read four and four, with ten lines commented out
-*       in VALIDATE_INPUT( ) and a note here saying the decision had not been
-*       made. It has been now - CJSMIG-687 Issue 4, "all fields should be
-*       mandatory" - so both ends were opened together. Change one end and
-*       the other has to move with it, or the dialog either promises an
-*       asterisk it does not enforce or refuses an OK it never marked.
-*
-*       THE HISTORY PICKER IS GONE, not commented out: "Use a previous
-*       declaration - field not required" (same ticket). HISTORY_OPTS( ),
-*       HISTORY_APPLY( ) and C_EVT_HIST are deliberately left in place - the
-*       same ticket asks for the legacy Search-from-History screen, which is
-*       a different control reading the same ChemicalHistorySet, and it will
-*       want them.
-        dialog_form(
-          io_ctx     = io_ctx
-          io_popup   = io_popup
-          iv_title   = 'Add Chemical'
-*         Two per row. "Alignment instead each row one filed, can have 2 or
-*         more field for better user experiences" - fourteen fields one to a
-*         row is a dialog nobody can see the bottom of.
-          iv_columns = 2
-          it_fields  = VALUE #(
-                                ( name = c_hs_pop           label = 'HS Code' required = abap_true
-                                  placeholder = 'e.g. 2933.99.90' )
-                                ( name = c_mat_pop          label = 'Material Name' required = abap_true )
-                                ( name = c_chem_pop         label = 'Chemical Name' required = abap_true )
-                                ( name = c_cas_no_pop       label = 'CAS Number' maxlen = 20 required = abap_true )
-                                ( name = c_chem_form_pop    label = 'Chemical Formula' required = abap_true )
-                                ( name = c_packaging_pop    label = 'Packing' required = abap_true )
-                                ( name = c_quantity_pop     label = 'Quantity' required = abap_true )
-                                ( name = c_gross_weight_pop label = 'Gross Weight' required = abap_true type = 'Number' )
-                                ( name = c_unit_pop         label = 'Unit' required = abap_true
-                                type = 'SELECT'
-                                options = VALUE #( ( key = 'GAL' text = 'Gallon' )
-                                                     ( key = 'KG'  text = 'Kilogram' )
-                                                     ( key = 'LIT' text = 'Liter' )
-                                                     ( key = 'MAT' text = 'Metric Ton' ) ) )
-                                ( name = c_invoice_pop      label = 'Invoice Number' required = abap_true )
-                                ( name = c_import_pop       label = 'Importing Country' shlp = 'H_T005' required = abap_true )
-                                ( name = c_exit_port_pop    label = 'Exit Port' required = abap_true )
-                                ( name = c_bol_pop          label = 'Bill of Lading' required = abap_true )
-                                ( name = c_tport_pop        label = 'Transport Details' required = abap_true )
-                              )
-          iv_ok_text = 'Add'
-          iv_ok_evt  = c_evt_ownok
-          iv_cxl_evt = c_evt_owncx ).
-    ENDCASE.
-  ENDMETHOD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>E018</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-697</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_CUSTOM_VALIDATE</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Same role-flag fix as E017</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_custom_validate.
-    rt = super-&gt;zif_rak_journey_logic~on_custom_validate( io_ctx  = io_ctx
-                                                          iv_step = iv_step ).
-    CASE iv_step.
-      WHEN 0.
-*       RE-DERIVED, NOT REFUSED.
-*
-*       PARTNER_OWNER/PARTNER_REP and PERMIT_YES/PERMIT_NO are not answers
-*       in their own right - they are WRITE_FLAGS( )'s projection of
-*       APPLICANT_ROLE and PERMIT_HELD, which are the fields the citizen
-*       actually fills in. This used to refuse the step whenever the role
-*       was set and its flags were not, with "Re-select Owner or
-*       Representative before continuing."
-*
-*       The citizen had already selected it. WRITE_FLAGS( ) only runs from
-*       ON_CHANGE( ), so any round trip that reinstates the model without
-*       raising a change on APPLICANT_ROLE - a backend read answering the
-*       step, the BP search coming back - leaves the role set and the flags
-*       blank. Re-selecting the same value raises no CHANGE either, so the
-*       one instruction the message gave could not clear it: the journey
-*       stopped at step 1. Reported on all three chemical journeys as
-*       "error showing we u select representative and search with owner EID
-*       details, not moving to next step".
-*
-*       Rewriting them is what the handler does at post time anyway -
-*       ON_BEFORE_POST( ) calls WRITE_FLAGS( ) before every post - so doing
-*       it here costs nothing and removes the only state that could block.
-        write_flags( io_ctx ).
-      WHEN 2.
-        DATA(ls_grid) = io_ctx-&gt;get_grid_data( c_grid ).
-        IF ls_grid-rows IS INITIAL.
-          APPEND VALUE #( type  = 'Error'
-*                          field = c_grid
-                          text  = `Add at least one material row.` ) TO rt.
-        ENDIF.
-      WHEN OTHERS.
-    ENDCASE.
-  ENDMETHOD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>E018</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-697</t>
-        </is>
-      </c>
-      <c r="C14" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_RENDER_POPUP</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Add Chemical: the fourteen required markers, and IV_COLUMNS = 2</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_render_popup.
-    super-&gt;zif_rak_journey_logic~on_render_popup(
-          io_ctx   = io_ctx
-          io_popup = io_popup
-          iv_id    = iv_id
-        ).
-**    CHECK iv_id = c_pop_mat.
-    CASE iv_id. "c_chem."
-      WHEN 'c_chem1'.
-*        render_own_popup( io_ctx = io_ctx io_popup = io_popup ).
-*        RETURN.
-      WHEN c_chem. "c_evt_details. "c_chem. "c_evt_details. " FOr F4 use this
-*       REQUIRED here is the marker only - DIALOG_FORM( ) sets it on the label
-*       and enforces nothing; a popup's enforcement is the handler's own, in the
-*       OK event. So this list mirrors WHEN c_evt_ownok exactly - now all
-*       fourteen marked and all fourteen tested, per CJSMIG-697 Issue 4 "all
-*       fields should be mandatory". Move one end and the other has to move
-*       with it.
-        dialog_form(
-          io_ctx     = io_ctx
-          io_popup   = io_popup
-          iv_title   = 'Add Chemical'
-*         Two per row. "Alignment instead each row one filed, can have 2 or
-*         more field for better user experiences" - same ticket.
-          iv_columns = 2
-          it_fields  = VALUE #(
-*                             The history picker stays out: "Use a previous
-*                             declaration - field not required". HISTORY_OPTS( )
-*                             and HISTORY_APPLY( ) are kept for the legacy
-*                             Search-from-History screen the same ticket asks
-*                             for, which is a different control.
-                                ( name = c_hs_code_pop          label = 'HS Code' required = abap_true
-                                  placeholder = 'e.g. 2933.99.90' )
-                                ( name = c_material_name_pop    label = 'Material Name' required = abap_true )
-                                ( name = c_chemical_name_pop    label = 'Chemical Name' required = abap_true )
-                                ( name = c_cas_pop              label = 'CAS Number' maxlen = 20 required = abap_true )
-                                ( name = c_chemical_formula_pop label = 'Chemical Formula' required = abap_true )
-                                ( name = c_packaging_pop        label = 'Packing' required = abap_true )
-                                ( name = c_quantity_pop         label = 'Quantity' required = abap_true )
-                                ( name = c_gross_weight_pop     label = 'Gross Weight' required = abap_true )
-                                ( name = c_uom_pop              label = 'UOM' type = 'SELECT' required = abap_true
-                                  options = VALUE #( ( key = 'GAL' text = 'Gallon' )
-                                                     ( key = 'KG'  text = 'Kilogram' )
-                                                     ( key = 'LIT' text = 'Liter' )
-                                                     ( key = 'MAT' text = 'Metric Ton' ) ) )
-                                ( name = c_invoice_pop          label = 'Invoice Number' required = abap_true )
-                                ( name = c_origin_pop           label = 'Country of Origin' shlp = 'H_T005' required = abap_true )
-                                ( name = c_end_user_pop         label = 'Point of Entrance' required = abap_true )
-                                ( name = c_bol_pop              label = 'Bill of Lading' required = abap_true )
-                                ( name = c_trans_comp           label = 'Transport Company' required = abap_true )
-                              )
-          iv_ok_text = 'Add'
-          iv_ok_evt  = c_evt_ownok
-          iv_cxl_evt = c_evt_owncx ).
-        RETURN.
-*        dialog_form(
-*          io_ctx     = io_ctx
-*          io_popup   = io_popup
-*          iv_title   = 'Add Chemical'
-*          it_fields  = VALUE #(
-*                                ( name = c_hs_code_pop          label = 'HS Code'  )
-*                                ( name = c_material_name_pop    label = 'Material Name' )
-*                                ( name = c_chemical_name_pop    label = 'Chemical Name' )
-*                                ( name = c_cas_pop              label = 'CAS Number' )
-*                                ( name = c_chemical_formula_pop label = 'Chemical Formula' )
-*                                ( name = c_packaging_pop        label = 'Packing' )
-*                                ( name = c_quantity_pop         label = 'Quantity'  )
-*                                ( name = c_gross_weight_pop     label = 'Gross Weight'  )
-*                                ( name = c_uom_pop              label = 'UOM'  )
-*                                ( name = c_invoice_pop          label = 'Invoice Number'  )
-*                                ( name = c_origin_pop           label = 'Country of Origin'  )
-*                                ( name = c_end_user_pop         label = 'Point of Entrance'  )
-*                                ( name = c_bol_pop              label = 'Bill of Lading'  )
-*                                ( name = c_trans_comp           label = 'Transport Company'  )
-*                              )
-*          iv_ok_text = 'Add'
-*          iv_ok_evt  = c_own_add ).
-      WHEN OTHERS.
-    ENDCASE.
-  ENDMETHOD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>E018</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>CJSMIG-697</t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
-        </is>
-      </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_POPUP_EVENT</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Add Chemical: all fourteen enforced on OK, and the dialog stays open when one fails</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_popup_event.
-    CALL METHOD super-&gt;zif_rak_journey_logic~on_popup_event
-      EXPORTING
-        io_ctx   = io_ctx
-        iv_id    = iv_id
-        iv_event = iv_event.
-    CASE iv_event.
-      WHEN c_evt_details.
-        chem_form_load( io_ctx ).          " no id = a new owner
-        io_ctx-&gt;open_popup( c_chem ).
-      WHEN c_evt_ownok. "'OWNER_ADD'. "
-*       Nothing here used to check any field - Add saved whatever was typed,
-*       blank fields included. All fourteen are now tested, mirroring the
-*       REQUIRED markers in ON_RENDER_POPUP( ) one for one.
-        IF io_ctx-&gt;get_val( c_hs_code_pop )          IS INITIAL
-           OR io_ctx-&gt;get_val( c_material_name_pop )    IS INITIAL
-           OR io_ctx-&gt;get_val( c_chemical_name_pop )    IS INITIAL
-           OR io_ctx-&gt;get_val( c_cas_pop )              IS INITIAL
-           OR io_ctx-&gt;get_val( c_chemical_formula_pop ) IS INITIAL
-           OR io_ctx-&gt;get_val( c_packaging_pop )     IS INITIAL
-           OR io_ctx-&gt;get_val( c_quantity_pop )      IS INITIAL
-           OR io_ctx-&gt;get_val( c_gross_weight_pop )  IS INITIAL
-           OR io_ctx-&gt;get_val( c_uom_pop )           IS INITIAL
-           OR io_ctx-&gt;get_val( c_invoice_pop )       IS INITIAL
-           OR io_ctx-&gt;get_val( c_origin_pop )        IS INITIAL
-           OR io_ctx-&gt;get_val( c_end_user_pop )      IS INITIAL
-           OR io_ctx-&gt;get_val( c_bol_pop )           IS INITIAL
-           OR io_ctx-&gt;get_val( c_trans_comp )        IS INITIAL.
-          io_ctx-&gt;add_msg( iv_type = 'Warning'
-                           iv_text = 'Kindly fill required details.' ).
-          RETURN.
-        ENDIF.
-        own_form_save( io_ctx ).
-        io_ctx-&gt;close_popup( ). "Close pop-up screen after adding data
-*      WHEN c_evt_hist.
-**       Fill the dialog from the chosen declaration and leave it OPEN - this
-**       shipment's own figures are still to type.
-*        history_apply( io_ctx ).
-      WHEN c_evt_owncx. "'CANCEL'. "
-        io_ctx-&gt;close_popup( ).
-*      WHEN c_evt_ownsr.
-*        own_search( io_ctx ).
-      WHEN OTHERS.
-*    "Edit Chemicals Details GRID
-        IF iv_event CP c_edit_pop.
-          own_edit( io_ctx = io_ctx iv_id = substring( val = iv_event off = 9 ) ).
-          io_ctx-&gt;open_popup( c_chem ).
-          RETURN.
-*     "Delete data from Chemicals Details GRID
-        ELSEIF iv_event CP c_DELETE_POP.
-          own_delete( io_ctx = io_ctx iv_id = substring( val = iv_event off = 8 ) ).
-          RETURN.
-        ENDIF.
-    ENDCASE.
-  ENDMETHOD.</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The journey's OWN class, not the framework. Read it, take it, or write your own - it is your service. Where a whole method is given it is the complete current method: replace the method body with it. Nothing here is pushed for anyone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>E025  ·  CJSMIG-703  ·  ZCL_E025_BEEKEEPING_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>see the code below   |   Applicant BP was written to the owner SEARCH field and then blanked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>* --- private section: the constant named the wrong field ------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>*   was:  constants C_LOGIN_BP type STRING value 'OWNER_BP' ##NO_TEXT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  constants C_LOGIN_BP type STRING value 'LOGIN_BP' ##NO_TEXT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>* --- ZIF_RAK_JOURNEY_LOGIC~ON_INIT, last line inside the IF -----------</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>*   was:  io_ctx-&gt;set_val( iv_name = 'OWNER_BP' iv_value = ' ' ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>*   'OWNER_BP' is the owner search box (see ON_SEARCH), not the applicant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  io_ctx-&gt;set_val( iv_name = c_owner_bp iv_value = ' ' ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>E026  ·  CJSMIG-704  ·  ZCL_E026_TREE_REMOVAL_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>see the code below   |   Applicant BP never reached LOGIN_BP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>* --- private section: add, leave C_LOGIN_BP exactly as it is ---------</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  constants C_APP_BP type STRING value 'LOGIN_BP' ##NO_TEXT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>* --- ZIF_RAK_JOURNEY_LOGIC~ON_INIT, straight after the existing line --</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    io_ctx-&gt;set_val( iv_name = c_login_bp iv_value = |{ lv_loginbp }| ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    io_ctx-&gt;set_val( iv_name = c_app_bp   iv_value = |{ lv_loginbp }| ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>E018  ·  CJSMIG-697  ·  ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>see the code below   |   The class had NO ACTIVE VERSION - a string constant does not take an empty literal, so every earlier fix was in the source and none of it was running</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>* --- private section --------------------------------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>*   was:  constants C_IMPEXP type STRING value ''.       &lt;- will not compile</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  constants C_IMPEXP type STRING value IS INITIAL ##NO_TEXT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>* Activate the class after this and re-test the whole journey - including the</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>* CX_SY_CONVERSION_NO_NUMBER on post, which may go with it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>E022  ·  CJSMIG-684  ·  ZCL_EPDA_E022_DEV_PROJ_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_INIT   |   Applicant details were written twice on ON_INIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_init.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>*CALL METHOD SUPER-&gt;ZIF_RAK_JOURNEY_LOGIC~ON_INIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>*  EXPORTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>*    IO_CTX =</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>*    .</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CALL METHOD super-&gt;zif_rak_journey_logic~on_init</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      EXPORTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        io_ctx = io_ctx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DATA: lv_loginbp TYPE bu_partner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    lv_loginbp       = CAST zcl_rak_journey_engine( io_ctx )-&gt;mv_loginbp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DATA(lv_rolebp)  = CAST zcl_rak_journey_engine( io_ctx )-&gt;mv_rolebp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DATA(lv_role)    = CAST zcl_rak_journey_engine( io_ctx )-&gt;mv_role. "Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    IF lv_loginbp IS NOT INITIAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      NEW zcl_ega_epda_fshry_handler_api( )-&gt;get_bp_details(</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        EXPORTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_bp_id      = lv_loginbp</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        IMPORTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          es_bp_details = DATA(ls_bp) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;set_val( iv_name = c_login_bp iv_value = |{ lv_loginbp }| ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="22" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="22" t="inlineStr">
+        <is>
+          <t>*     WRITTEN ONCE. C_PARTNER_NAME is 'APP_NAME' and C_PARTNER_ID is</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
+          <t>*     'APP_ID', and both were then written a SECOND time below this IF, under</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>*     a different language rule - so the two disagreed and the later one won.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>*     The pair below the IF was also outside this guard, so a launch with no</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="22" t="inlineStr">
+        <is>
+          <t>*     login partner blanked the applicant's name and ID rather than leaving</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>*     them alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>*     The rule kept is the one that degrades: an Arabic session with no</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="22" t="inlineStr">
+        <is>
+          <t>*     Arabic name on the partner record falls back to the English name</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="22" t="inlineStr">
+        <is>
+          <t>*     rather than showing an empty applicant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;set_val( iv_name  = c_partner_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                       iv_value = COND #( WHEN sy-langu &lt;&gt; c_lang_en AND ls_bp-bp_name_ar IS NOT INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                          THEN CONV string( ls_bp-bp_name_ar )</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                          ELSE CONV string( ls_bp-bp_name ) ) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="22" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;set_val( iv_name = c_partner_id iv_value = CONV #( ls_bp-emirates_id ) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="22" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;set_val( iv_name = c_partner_mobile iv_value = CONV #( ls_bp-mobile_number ) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;set_val( iv_name = c_partner_email iv_value = CONV #( ls_bp-email_address ) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="22" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="22" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;set_val( iv_name = c_applicanttype iv_value = |{ lv_role }| ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="22" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="22" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="22" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="20" t="inlineStr">
+        <is>
+          <t>E022 E026 E027 D021 D014gv  ·  CJSMIG-684 / 704  ·  six classes - see the code</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="21" t="inlineStr">
+        <is>
+          <t>see the code below   |   The applicant's own partner never reached LOGIN_BP, the field every other journey and the record model use. Additive: the existing OWNER_BP write is left alone, so nothing that works today changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="22" t="inlineStr">
+        <is>
+          <t>* Applies to ZCL_EPDA_E022_DEV_PROJ_LOGIC, ZCL_E026_TREE_REMOVAL_LOGIC,</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="22" t="inlineStr">
+        <is>
+          <t>* ZCL_E027_VICE_CAPTAIN_LOGIC, ZCL_D021_MOD_SCHOOL_FEE_LOGIC and</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="22" t="inlineStr">
+        <is>
+          <t>* ZCL_D014_STAFF_GOLD_VISA_LOGIC - all five declare C_LOGIN_BP as 'OWNER_BP'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="22" t="inlineStr">
+        <is>
+          <t>* E025 is the exception and has its own row above: there OWNER_BP is the owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="22" t="inlineStr">
+        <is>
+          <t>* SEARCH box, so the constant itself has to be corrected, not added to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="22" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="22" t="inlineStr">
+        <is>
+          <t>* --- private section: ADD this. Leave C_LOGIN_BP exactly as it is. ----</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  constants C_APP_BP type STRING value 'LOGIN_BP' ##NO_TEXT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="22" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="22" t="inlineStr">
+        <is>
+          <t>* --- ON_INIT: ADD the second line under the existing first one. -------</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    io_ctx-&gt;set_val( iv_name = c_login_bp iv_value = |{ lv_loginbp }| ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    io_ctx-&gt;set_val( iv_name = c_app_bp   iv_value = |{ lv_loginbp }| ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="20" t="inlineStr">
+        <is>
+          <t>E017  ·  CJSMIG-687  ·  ZCL_E017_NOC_EXP_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="21" t="inlineStr">
+        <is>
+          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_CUSTOM_VALIDATE   |   Step 0 refused whenever the role flags disagreed with APPLICANT_ROLE - re-derived now instead of refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_custom_validate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="22" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    rt = super-&gt;zif_rak_journey_logic~on_custom_validate( io_ctx  = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                          iv_step = iv_step ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="22" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CASE iv_step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="22" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="22" t="inlineStr">
+        <is>
+          <t>*       RE-DERIVED, NOT REFUSED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="22" t="inlineStr">
+        <is>
+          <t>*       PARTNER_OWNER/PARTNER_REP and PERMIT_YES/PERMIT_NO are not answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="22" t="inlineStr">
+        <is>
+          <t>*       in their own right - they are WRITE_FLAGS( )'s projection of</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="22" t="inlineStr">
+        <is>
+          <t>*       APPLICANT_ROLE and PERMIT_HELD, which are the fields the citizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="22" t="inlineStr">
+        <is>
+          <t>*       actually fills in. This used to refuse the step whenever the role</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="22" t="inlineStr">
+        <is>
+          <t>*       was set and its flags were not, with "Re-select Owner or</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="22" t="inlineStr">
+        <is>
+          <t>*       Representative before continuing."</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="22" t="inlineStr">
+        <is>
+          <t>*       The citizen had already selected it. WRITE_FLAGS( ) only runs from</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="22" t="inlineStr">
+        <is>
+          <t>*       ON_CHANGE( ), so any round trip that reinstates the model without</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="22" t="inlineStr">
+        <is>
+          <t>*       raising a change on APPLICANT_ROLE - a backend read answering the</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="22" t="inlineStr">
+        <is>
+          <t>*       step, the BP search coming back - leaves the role set and the flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="22" t="inlineStr">
+        <is>
+          <t>*       blank. Re-selecting the same value raises no CHANGE either, so the</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="22" t="inlineStr">
+        <is>
+          <t>*       one instruction the message gave could not clear it: the journey</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="22" t="inlineStr">
+        <is>
+          <t>*       stopped at step 1. Reported on all three chemical journeys as</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="22" t="inlineStr">
+        <is>
+          <t>*       "error showing we u select representative and search with owner EID</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="22" t="inlineStr">
+        <is>
+          <t>*       details, not moving to next step".</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="22" t="inlineStr">
+        <is>
+          <t>*       Rewriting them is what the handler does at post time anyway -</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="22" t="inlineStr">
+        <is>
+          <t>*       ON_BEFORE_POST( ) calls WRITE_FLAGS( ) before every post - so doing</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="22" t="inlineStr">
+        <is>
+          <t>*       it here costs nothing and removes the only state that could block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        write_flags( io_ctx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="22" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        DATA(ls_grid) = io_ctx-&gt;get_grid_data( c_grid ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        IF ls_grid-rows IS INITIAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          APPEND VALUE #( type  = 'Error' "field = c_grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                          text  = `Add at least one chemical row.` ) TO rt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ENDIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="22" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN OTHERS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDCASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="22" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1">
+      <c r="A150" s="20" t="inlineStr">
+        <is>
+          <t>E017  ·  CJSMIG-687  ·  ZCL_E017_NOC_EXP_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="30" customHeight="1">
+      <c r="A151" s="21" t="inlineStr">
+        <is>
+          <t>METHOD VALIDATE_INPUT   |   Add Chemical: all fourteen fields enforced. Ten of the checks were commented out</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD validate_input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="22" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="22" t="inlineStr">
+        <is>
+          <t>*   ALL FOURTEEN, mirroring the REQUIRED markers in ON_RENDER_POPUP( ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="22" t="inlineStr">
+        <is>
+          <t>*   Ten of these were commented out; CJSMIG-687 Issue 4 settled it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    IF io_ctx-&gt;get_val( c_hs_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_mat_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_chem_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_cas_no_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_chem_form_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_packaging_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_quantity_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_gross_weight_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_unit_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_bol_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_exit_port_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_import_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             OR io_ctx-&gt;get_val( c_tport_pop ) IS INITIAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="22" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="22" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx-&gt;add_msg( iv_type = 'Warning'</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                       iv_text = 'Kindly fill required details.' ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="22" t="inlineStr">
+        <is>
+          <t>*     RV_OK stays FALSE. This used to return nothing at all, and ON_POPUP_EVENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="22" t="inlineStr">
+        <is>
+          <t>*     called POPULATE_GRID( ) and CLOSE_POPUP( ) straight afterwards whatever</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="22" t="inlineStr">
+        <is>
+          <t>*     happened here - so a blank row was added to the grid and the dialog shut,</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="22" t="inlineStr">
+        <is>
+          <t>*     with only a warning toast to say otherwise. The verdict has to reach the</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="22" t="inlineStr">
+        <is>
+          <t>*     caller for the message to mean anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="22" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    rv_ok = abap_true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="22" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="A185" s="20" t="inlineStr">
+        <is>
+          <t>E017  ·  CJSMIG-687  ·  ZCL_E017_NOC_EXP_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="21" t="inlineStr">
+        <is>
+          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_RENDER_POPUP   |   Add Chemical: the fourteen required markers, and IV_COLUMNS = 2 for the two-column dialog</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_render_popup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    super-&gt;zif_rak_journey_logic~on_render_popup(</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_ctx   = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      io_popup = io_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      iv_id    = iv_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="22" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CASE iv_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="22" t="inlineStr">
+        <is>
+          <t>*  "On click of ADD Chemical button</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN c_open_popup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="22" t="inlineStr">
+        <is>
+          <t>*        render_own_popup( io_ctx = io_ctx io_popup = io_popup ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="22" t="inlineStr">
+        <is>
+          <t>*        RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="22" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="22" t="inlineStr">
+        <is>
+          <t>*       REQUIRED here is the marker only - DIALOG_FORM( ) sets it on the label</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="22" t="inlineStr">
+        <is>
+          <t>*       and enforces nothing; a popup's enforcement is the handler's, in</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="22" t="inlineStr">
+        <is>
+          <t>*       VALIDATE_INPUT( ). So this list has to mirror that method exactly,</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="22" t="inlineStr">
+        <is>
+          <t>*       and now does: all fourteen marked, all fourteen checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="22" t="inlineStr">
+        <is>
+          <t>*       That mirror used to read four and four, with ten lines commented out</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="22" t="inlineStr">
+        <is>
+          <t>*       in VALIDATE_INPUT( ) and a note here saying the decision had not been</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="22" t="inlineStr">
+        <is>
+          <t>*       made. It has been now - CJSMIG-687 Issue 4, "all fields should be</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="22" t="inlineStr">
+        <is>
+          <t>*       mandatory" - so both ends were opened together. Change one end and</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="22" t="inlineStr">
+        <is>
+          <t>*       the other has to move with it, or the dialog either promises an</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="22" t="inlineStr">
+        <is>
+          <t>*       asterisk it does not enforce or refuses an OK it never marked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="22" t="inlineStr">
+        <is>
+          <t>*       THE HISTORY PICKER IS GONE, not commented out: "Use a previous</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="22" t="inlineStr">
+        <is>
+          <t>*       declaration - field not required" (same ticket). HISTORY_OPTS( ),</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="22" t="inlineStr">
+        <is>
+          <t>*       HISTORY_APPLY( ) and C_EVT_HIST are deliberately left in place - the</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="22" t="inlineStr">
+        <is>
+          <t>*       same ticket asks for the legacy Search-from-History screen, which is</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="22" t="inlineStr">
+        <is>
+          <t>*       a different control reading the same ChemicalHistorySet, and it will</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="22" t="inlineStr">
+        <is>
+          <t>*       want them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        dialog_form(</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_ctx     = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_popup   = io_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_title   = 'Add Chemical'</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="22" t="inlineStr">
+        <is>
+          <t>*         Two per row. "Alignment instead each row one filed, can have 2 or</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="22" t="inlineStr">
+        <is>
+          <t>*         more field for better user experiences" - fourteen fields one to a</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="22" t="inlineStr">
+        <is>
+          <t>*         row is a dialog nobody can see the bottom of.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_columns = 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          it_fields  = VALUE #(</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_hs_pop           label = 'HS Code' required = abap_true</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  placeholder = 'e.g. 2933.99.90' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_mat_pop          label = 'Material Name' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_chem_pop         label = 'Chemical Name' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_cas_no_pop       label = 'CAS Number' maxlen = 20 required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_chem_form_pop    label = 'Chemical Formula' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_packaging_pop    label = 'Packing' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_quantity_pop     label = 'Quantity' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_gross_weight_pop label = 'Gross Weight' required = abap_true type = 'Number' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_unit_pop         label = 'Unit' required = abap_true</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                type = 'SELECT'</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                options = VALUE #( ( key = 'GAL' text = 'Gallon' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                     ( key = 'KG'  text = 'Kilogram' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                     ( key = 'LIT' text = 'Liter' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                     ( key = 'MAT' text = 'Metric Ton' ) ) )</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_invoice_pop      label = 'Invoice Number' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_import_pop       label = 'Importing Country' shlp = 'H_T005' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_exit_port_pop    label = 'Exit Port' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_bol_pop          label = 'Bill of Lading' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_tport_pop        label = 'Transport Details' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                              )</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_ok_text = 'Add'</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_ok_evt  = c_evt_ownok</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_cxl_evt = c_evt_owncx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDCASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="20" customHeight="1">
+      <c r="A254" s="20" t="inlineStr">
+        <is>
+          <t>E018  ·  CJSMIG-697  ·  ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="30" customHeight="1">
+      <c r="A255" s="21" t="inlineStr">
+        <is>
+          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_CUSTOM_VALIDATE   |   Same role-flag fix as E017</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_custom_validate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    rt = super-&gt;zif_rak_journey_logic~on_custom_validate( io_ctx  = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                          iv_step = iv_step ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="22" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CASE iv_step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="22" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="22" t="inlineStr">
+        <is>
+          <t>*       RE-DERIVED, NOT REFUSED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="22" t="inlineStr">
+        <is>
+          <t>*       PARTNER_OWNER/PARTNER_REP and PERMIT_YES/PERMIT_NO are not answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="22" t="inlineStr">
+        <is>
+          <t>*       in their own right - they are WRITE_FLAGS( )'s projection of</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="22" t="inlineStr">
+        <is>
+          <t>*       APPLICANT_ROLE and PERMIT_HELD, which are the fields the citizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="22" t="inlineStr">
+        <is>
+          <t>*       actually fills in. This used to refuse the step whenever the role</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="22" t="inlineStr">
+        <is>
+          <t>*       was set and its flags were not, with "Re-select Owner or</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="22" t="inlineStr">
+        <is>
+          <t>*       Representative before continuing."</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="22" t="inlineStr">
+        <is>
+          <t>*       The citizen had already selected it. WRITE_FLAGS( ) only runs from</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="22" t="inlineStr">
+        <is>
+          <t>*       ON_CHANGE( ), so any round trip that reinstates the model without</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="22" t="inlineStr">
+        <is>
+          <t>*       raising a change on APPLICANT_ROLE - a backend read answering the</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="22" t="inlineStr">
+        <is>
+          <t>*       step, the BP search coming back - leaves the role set and the flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="22" t="inlineStr">
+        <is>
+          <t>*       blank. Re-selecting the same value raises no CHANGE either, so the</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="22" t="inlineStr">
+        <is>
+          <t>*       one instruction the message gave could not clear it: the journey</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="22" t="inlineStr">
+        <is>
+          <t>*       stopped at step 1. Reported on all three chemical journeys as</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="22" t="inlineStr">
+        <is>
+          <t>*       "error showing we u select representative and search with owner EID</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="22" t="inlineStr">
+        <is>
+          <t>*       details, not moving to next step".</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="22" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="22" t="inlineStr">
+        <is>
+          <t>*       Rewriting them is what the handler does at post time anyway -</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="22" t="inlineStr">
+        <is>
+          <t>*       ON_BEFORE_POST( ) calls WRITE_FLAGS( ) before every post - so doing</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="22" t="inlineStr">
+        <is>
+          <t>*       it here costs nothing and removes the only state that could block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        write_flags( io_ctx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="22" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        DATA(ls_grid) = io_ctx-&gt;get_grid_data( c_grid ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        IF ls_grid-rows IS INITIAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          APPEND VALUE #( type  = 'Error'</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="22" t="inlineStr">
+        <is>
+          <t>*                          field = c_grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                          text  = `Add at least one material row.` ) TO rt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ENDIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="22" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN OTHERS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDCASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="22" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="20" customHeight="1">
+      <c r="A300" s="20" t="inlineStr">
+        <is>
+          <t>E018  ·  CJSMIG-697  ·  ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="30" customHeight="1">
+      <c r="A301" s="21" t="inlineStr">
+        <is>
+          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_RENDER_POPUP   |   Add Chemical: the fourteen required markers, and IV_COLUMNS = 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_render_popup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="22" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    super-&gt;zif_rak_journey_logic~on_render_popup(</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_ctx   = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_popup = io_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_id    = iv_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="22" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="22" t="inlineStr">
+        <is>
+          <t>**    CHECK iv_id = c_pop_mat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CASE iv_id. "c_chem."</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN 'c_chem1'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="22" t="inlineStr">
+        <is>
+          <t>*        render_own_popup( io_ctx = io_ctx io_popup = io_popup ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="22" t="inlineStr">
+        <is>
+          <t>*        RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN c_chem. "c_evt_details. "c_chem. "c_evt_details. " FOr F4 use this</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="22" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="22" t="inlineStr">
+        <is>
+          <t>*       REQUIRED here is the marker only - DIALOG_FORM( ) sets it on the label</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="22" t="inlineStr">
+        <is>
+          <t>*       and enforces nothing; a popup's enforcement is the handler's own, in the</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="22" t="inlineStr">
+        <is>
+          <t>*       OK event. So this list mirrors WHEN c_evt_ownok exactly - now all</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="22" t="inlineStr">
+        <is>
+          <t>*       fourteen marked and all fourteen tested, per CJSMIG-697 Issue 4 "all</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="22" t="inlineStr">
+        <is>
+          <t>*       fields should be mandatory". Move one end and the other has to move</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="22" t="inlineStr">
+        <is>
+          <t>*       with it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        dialog_form(</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_ctx     = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_popup   = io_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_title   = 'Add Chemical'</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="22" t="inlineStr">
+        <is>
+          <t>*         Two per row. "Alignment instead each row one filed, can have 2 or</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="22" t="inlineStr">
+        <is>
+          <t>*         more field for better user experiences" - same ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_columns = 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          it_fields  = VALUE #(</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="22" t="inlineStr">
+        <is>
+          <t>*                             The history picker stays out: "Use a previous</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="22" t="inlineStr">
+        <is>
+          <t>*                             declaration - field not required". HISTORY_OPTS( )</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="22" t="inlineStr">
+        <is>
+          <t>*                             and HISTORY_APPLY( ) are kept for the legacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="22" t="inlineStr">
+        <is>
+          <t>*                             Search-from-History screen the same ticket asks</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="22" t="inlineStr">
+        <is>
+          <t>*                             for, which is a different control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_hs_code_pop          label = 'HS Code' required = abap_true</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  placeholder = 'e.g. 2933.99.90' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_material_name_pop    label = 'Material Name' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_chemical_name_pop    label = 'Chemical Name' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_cas_pop              label = 'CAS Number' maxlen = 20 required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_chemical_formula_pop label = 'Chemical Formula' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_packaging_pop        label = 'Packing' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_quantity_pop         label = 'Quantity' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_gross_weight_pop     label = 'Gross Weight' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_uom_pop              label = 'UOM' type = 'SELECT' required = abap_true</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  options = VALUE #( ( key = 'GAL' text = 'Gallon' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                     ( key = 'KG'  text = 'Kilogram' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                     ( key = 'LIT' text = 'Liter' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                     ( key = 'MAT' text = 'Metric Ton' ) ) )</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="22" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_invoice_pop          label = 'Invoice Number' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_origin_pop           label = 'Country of Origin' shlp = 'H_T005' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_end_user_pop         label = 'Point of Entrance' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_bol_pop              label = 'Bill of Lading' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ( name = c_trans_comp           label = 'Transport Company' required = abap_true )</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                              )</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="22" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_ok_text = 'Add'</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_ok_evt  = c_evt_ownok</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          iv_cxl_evt = c_evt_owncx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="22" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="22" t="inlineStr">
+        <is>
+          <t>*        dialog_form(</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="22" t="inlineStr">
+        <is>
+          <t>*          io_ctx     = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="22" t="inlineStr">
+        <is>
+          <t>*          io_popup   = io_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="22" t="inlineStr">
+        <is>
+          <t>*          iv_title   = 'Add Chemical'</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="22" t="inlineStr">
+        <is>
+          <t>*          it_fields  = VALUE #(</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_hs_code_pop          label = 'HS Code'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_material_name_pop    label = 'Material Name' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_chemical_name_pop    label = 'Chemical Name' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_cas_pop              label = 'CAS Number' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_chemical_formula_pop label = 'Chemical Formula' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_packaging_pop        label = 'Packing' )</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_quantity_pop         label = 'Quantity'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_gross_weight_pop     label = 'Gross Weight'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_uom_pop              label = 'UOM'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_invoice_pop          label = 'Invoice Number'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_origin_pop           label = 'Country of Origin'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_end_user_pop         label = 'Point of Entrance'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_bol_pop              label = 'Bill of Lading'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="22" t="inlineStr">
+        <is>
+          <t>*                                ( name = c_trans_comp           label = 'Transport Company'  )</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="22" t="inlineStr">
+        <is>
+          <t>*                              )</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="22" t="inlineStr">
+        <is>
+          <t>*          iv_ok_text = 'Add'</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="22" t="inlineStr">
+        <is>
+          <t>*          iv_ok_evt  = c_own_add ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="22" t="n"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN OTHERS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDCASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="22" t="n"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="20" customHeight="1">
+      <c r="A391" s="20" t="inlineStr">
+        <is>
+          <t>E018  ·  CJSMIG-697  ·  ZCL_E018_NOC_TRANS_CHEM_LOGIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="30" customHeight="1">
+      <c r="A392" s="21" t="inlineStr">
+        <is>
+          <t>METHOD ZIF_RAK_JOURNEY_LOGIC~ON_POPUP_EVENT   |   Add Chemical: all fourteen enforced on OK, and the dialog stays open when one fails</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  METHOD zif_rak_journey_logic~on_popup_event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="22" t="n"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="22" t="n"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="22" t="n"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CALL METHOD super-&gt;zif_rak_journey_logic~on_popup_event</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      EXPORTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        io_ctx   = io_ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        iv_id    = iv_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        iv_event = iv_event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="22" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CASE iv_event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN c_evt_details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        chem_form_load( io_ctx ).          " no id = a new owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        io_ctx-&gt;open_popup( c_chem ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="22" t="n"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN c_evt_ownok. "'OWNER_ADD'. "</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="22" t="inlineStr">
+        <is>
+          <t>*       Nothing here used to check any field - Add saved whatever was typed,</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="22" t="inlineStr">
+        <is>
+          <t>*       blank fields included. All fourteen are now tested, mirroring the</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="22" t="inlineStr">
+        <is>
+          <t>*       REQUIRED markers in ON_RENDER_POPUP( ) one for one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        IF io_ctx-&gt;get_val( c_hs_code_pop )          IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_material_name_pop )    IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_chemical_name_pop )    IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_cas_pop )              IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_chemical_formula_pop ) IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_packaging_pop )     IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_quantity_pop )      IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_gross_weight_pop )  IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_uom_pop )           IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_invoice_pop )       IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_origin_pop )        IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_end_user_pop )      IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_bol_pop )           IS INITIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           OR io_ctx-&gt;get_val( c_trans_comp )        IS INITIAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_ctx-&gt;add_msg( iv_type = 'Warning'</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                           iv_text = 'Kindly fill required details.' ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ENDIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="22" t="n"/>
+    </row>
+    <row r="431">
+      <c r="A431" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        own_form_save( io_ctx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        io_ctx-&gt;close_popup( ). "Close pop-up screen after adding data</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="22" t="n"/>
+    </row>
+    <row r="434">
+      <c r="A434" s="22" t="n"/>
+    </row>
+    <row r="435">
+      <c r="A435" s="22" t="inlineStr">
+        <is>
+          <t>*      WHEN c_evt_hist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="22" t="inlineStr">
+        <is>
+          <t>**       Fill the dialog from the chosen declaration and leave it OPEN - this</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="22" t="inlineStr">
+        <is>
+          <t>**       shipment's own figures are still to type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="22" t="inlineStr">
+        <is>
+          <t>*        history_apply( io_ctx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="22" t="n"/>
+    </row>
+    <row r="440">
+      <c r="A440" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN c_evt_owncx. "'CANCEL'. "</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        io_ctx-&gt;close_popup( ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="22" t="n"/>
+    </row>
+    <row r="443">
+      <c r="A443" s="22" t="inlineStr">
+        <is>
+          <t>*      WHEN c_evt_ownsr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="22" t="inlineStr">
+        <is>
+          <t>*        own_search( io_ctx ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="22" t="n"/>
+    </row>
+    <row r="446">
+      <c r="A446" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      WHEN OTHERS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="22" t="inlineStr">
+        <is>
+          <t>*    "Edit Chemicals Details GRID</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        IF iv_event CP c_edit_pop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          own_edit( io_ctx = io_ctx iv_id = substring( val = iv_event off = 9 ) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          io_ctx-&gt;open_popup( c_chem ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="22" t="inlineStr">
+        <is>
+          <t>*     "Delete data from Chemicals Details GRID</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ELSEIF iv_event CP c_DELETE_POP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          own_delete( io_ctx = io_ctx iv_id = substring( val = iv_event off = 8 ) ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          RETURN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ENDIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="22" t="n"/>
+    </row>
+    <row r="458">
+      <c r="A458" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ENDCASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENDMETHOD.</t>
         </is>
       </c>
     </row>

</xml_diff>